<commit_message>
built a simple web UI to streamline our ADVP curation workflow.
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table3_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table3_v1.xlsx
@@ -780,7 +780,7 @@
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>DSG2</t>
+          <t>DLGAP1</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>DSG2</t>
+          <t>NETO1</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>EID2B</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>CD2AP</t>
+          <t>AK9</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>CD33</t>
+          <t>IER2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy locahhost to Render
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table3_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table3_v1.xlsx
@@ -672,27 +672,27 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>74046</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -720,12 +720,12 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -808,27 +808,27 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>74046</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -856,12 +856,12 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -944,27 +944,27 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>74046</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
@@ -992,12 +992,12 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1080,27 +1080,27 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>74046</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -1128,12 +1128,12 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1216,27 +1216,27 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>74046</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -1264,12 +1264,12 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>

</xml_diff>

<commit_message>
Allow the use of either PMCID or link with PMCID or pdf file
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table3_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table3_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AT6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,7 +516,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Imputation_simple2</t>
+          <t>Imputation</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -663,7 +663,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>rs8093731</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -678,194 +678,82 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>T00003</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['Meta-analysis', 'Discovery', 'IGAP']</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>['Imaging']</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>['logistic regression (with covariates)']</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>Meta-analysis + IGAP + Discovery</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>SNP-based</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>['74046']</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>ADSP + UKBB + ADNI + ADGC + UKBEC + IGAP + CHARGE + NABEC</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>['1000 Genomes', 'Haplotype Reference Consortium', 'TOPMed', 'UK10K']</t>
+          <t>UK10K + 1000 Genomes + Haplotype Reference Consortium + TOPMed</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>['European', '1000 Genomes EUR', 'ADGC', 'ADSP', 'IGAP']</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>ADSP + European + ADGC + IGAP + 1000 Genomes EUR</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>Alzheimer's disease + AD</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>rs8093731</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="n">
+        <v>1.36e-08</v>
+      </c>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="AL2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr">
         <is>
           <t>30448613</t>
@@ -874,17 +762,481 @@
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>Table 3</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>30448613_table3.xlsx</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>DLGAP1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rs8093731</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>30448613_table3_R00002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>30448613_table3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>T00003</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Meta-analysis + IGAP + Discovery</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>ADSP + UKBB + ADNI + ADGC + UKBEC + IGAP + CHARGE + NABEC</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>UK10K + 1000 Genomes + Haplotype Reference Consortium + TOPMed</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>ADSP + European + ADGC + IGAP + 1000 Genomes EUR</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Alzheimer's disease + AD</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>rs8093731</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="n">
+        <v>1.11e-05</v>
+      </c>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="AL3" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>Table 3</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>30448613_table3.xlsx</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>NETO1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>rs4147929</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>30448613_table3_R00003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>30448613_table3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>T00003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Meta-analysis + IGAP + Discovery</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>ADSP + UKBB + ADNI + ADGC + UKBEC + IGAP + CHARGE + NABEC</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>UK10K + 1000 Genomes + Haplotype Reference Consortium + TOPMed</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>ADSP + European + ADGC + IGAP + 1000 Genomes EUR</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Alzheimer's disease + AD</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>rs4147929</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="n">
+        <v>3.94e-06</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>Table 3</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>30448613_table3.xlsx</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>EID2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>rs10948363</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>30448613_table3_R00004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>30448613_table3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>T00003</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Meta-analysis + IGAP + Discovery</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>ADSP + UKBB + ADNI + ADGC + UKBEC + IGAP + CHARGE + NABEC</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>UK10K + 1000 Genomes + Haplotype Reference Consortium + TOPMed</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>ADSP + European + ADGC + IGAP + 1000 Genomes EUR</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Alzheimer's disease + AD</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>rs10948363</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="n">
+        <v>1.64e-05</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="AL5" t="n">
+        <v>0.343</v>
+      </c>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>Table 3</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>30448613_table3.xlsx</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>AK9</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rs3865444</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>30448613_table3_R00005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>30448613_table3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>T00003</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Meta-analysis + IGAP + Discovery</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ADSP + UKBB + ADNI + ADGC + UKBEC + IGAP + CHARGE + NABEC</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>UK10K + 1000 Genomes + Haplotype Reference Consortium + TOPMed</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>ADSP + European + ADGC + IGAP + 1000 Genomes EUR</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Alzheimer's disease + AD</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>rs3865444</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="n">
+        <v>1.96e-05</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="AL6" t="n">
+        <v>-0.255</v>
+      </c>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>Table 3</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>30448613_table3.xlsx</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>IER2</t>
         </is>
       </c>
     </row>

</xml_diff>